<commit_message>
v40 study: F4=F6 merge (same child, different id on PC vs paper), I-50 gaze does not explain sex interaction, results:html export script
- make_mapping.py: ALIAS F4->F6, single exclusion entry (8 excluded, 55 effective participants); classify_order.py applies alias (F6 now one ANOMALO-II row with F4's gaze)
- INSIGHTS: I-51 (merge documented as inference), I-50 (M/F gaze patterns nearly identical; comprehension benefit does not follow attention shift), I-17/I-20 updated, section D hypotheses all resolved
- package.json: npm run results:html (nbconvert export of the notebook, executed fresh)
- cohort of 48 and all main results unchanged

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/study/mappatura_soggetti.xlsx
+++ b/study/mappatura_soggetti.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1598,31 +1598,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F4</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>somministrazione anomala (images+images)</t>
-        </is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f> F4 nel gaze (stesso bambino); somministrazione anomala (images+images)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>F6</t>
+          <t>F10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>nessun gaze: ordine non verificabile</t>
+          <t>gaze parziale: ordine non verificabile</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1634,22 +1633,10 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>F25</t>
+          <t>F35</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
-        <is>
-          <t>gaze parziale: ordine non verificabile</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>F35</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
         <is>
           <t>somministrazione anomala (text+text)</t>
         </is>

</xml_diff>